<commit_message>
Updating deadlines and syllabus
</commit_message>
<xml_diff>
--- a/files/schedule_modules.xlsx
+++ b/files/schedule_modules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jessicacooperstone/git/rdataviz/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E585AACF-C814-8C42-B124-3E139AA782B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC4A8C7-1E71-CF4D-84CB-D36E5B9D68E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20980" yWindow="1900" windowWidth="28800" windowHeight="16360" activeTab="1" xr2:uid="{21EBE61F-A4F0-3D45-865A-9EB87E85AA6A}"/>
+    <workbookView xWindow="17480" yWindow="2380" windowWidth="28800" windowHeight="16360" activeTab="2" xr2:uid="{21EBE61F-A4F0-3D45-865A-9EB87E85AA6A}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="67">
   <si>
     <t>Principles of data visualization</t>
   </si>
@@ -224,6 +224,27 @@
   </si>
   <si>
     <t>ggplot extension packages (asynchronous)</t>
+  </si>
+  <si>
+    <t>Monday, September 7, 2026</t>
+  </si>
+  <si>
+    <t>Tuesday, October 13, 2026</t>
+  </si>
+  <si>
+    <t>Tuesday, November 3, 2026</t>
+  </si>
+  <si>
+    <t>Tuesday, December 8, 2026</t>
+  </si>
+  <si>
+    <t>Tuesday, November 10, 2026</t>
+  </si>
+  <si>
+    <t>Sunday, December 13, 2026</t>
+  </si>
+  <si>
+    <t>due_date_paste</t>
   </si>
 </sst>
 </file>
@@ -232,7 +253,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
-    <numFmt numFmtId="167" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -269,7 +290,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1056,7 +1077,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7EACCAF-8C8B-E146-ABA1-005F5C4A7B4F}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.33203125" bestFit="1" customWidth="1"/>
@@ -1064,31 +1085,40 @@
     <col min="3" max="3" width="22.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>26</v>
       </c>
       <c r="B1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>42</v>
       </c>
       <c r="B3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -1096,8 +1126,11 @@
         <f>Schedule_date_2026!B4 + -1</f>
         <v>46272</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -1105,8 +1138,11 @@
         <f>Schedule_date_2026!B9</f>
         <v>46308</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -1114,8 +1150,11 @@
         <f>Schedule_date_2026!B12</f>
         <v>46329</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1123,8 +1162,11 @@
         <f>Schedule_date_2026!B17</f>
         <v>46364</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -1132,14 +1174,20 @@
         <f>Schedule_date_2026!B13</f>
         <v>46336</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>32</v>
       </c>
       <c r="B9" s="5">
         <f>Schedule_date_2026!B17+5</f>
         <v>46369</v>
+      </c>
+      <c r="C9" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>